<commit_message>
Changed model - haiku 5.5
</commit_message>
<xml_diff>
--- a/Policy_Agent_Test_Results_v2.xlsx
+++ b/Policy_Agent_Test_Results_v2.xlsx
@@ -1195,7 +1195,7 @@
       </c>
       <c r="I8" s="71" t="inlineStr">
         <is>
-          <t>8 days, Sec 2.2, no ID asked. Omitted the 'certificate after 2 days' detail.</t>
+          <t>8 days, certificate after 2 consecutive days, Sec 2.2. No ID asked.</t>
         </is>
       </c>
     </row>
@@ -1318,7 +1318,7 @@
       </c>
       <c r="I11" s="71" t="inlineStr">
         <is>
-          <t>Up to 30,000/yr, manager approval first, Sec 4.3. No ID asked (failed last run).</t>
+          <t>Up to 30,000/yr, manager approval before enrolling, Sec 4.3. No ID asked.</t>
         </is>
       </c>
     </row>
@@ -1359,7 +1359,7 @@
       </c>
       <c r="I12" s="71" t="inlineStr">
         <is>
-          <t>By 15 June, Sec 3.2. No ID asked (failed last run).</t>
+          <t>By 15 June, Sec 3.2. No ID asked.</t>
         </is>
       </c>
     </row>
@@ -1400,7 +1400,7 @@
       </c>
       <c r="I13" s="71" t="inlineStr">
         <is>
-          <t>Within 45 days, Sec 7.2.</t>
+          <t>Within 45 days of last working day, Sec 7.2.</t>
         </is>
       </c>
     </row>
@@ -1431,17 +1431,17 @@
       </c>
       <c r="G14" s="70" t="inlineStr">
         <is>
-          <t>✓</t>
+          <t>☐</t>
         </is>
       </c>
       <c r="H14" s="70" t="inlineStr">
         <is>
-          <t>☐</t>
+          <t>❌</t>
         </is>
       </c>
       <c r="I14" s="71" t="inlineStr">
         <is>
-          <t>Both: 30 days probation / 60 days permanent, Sec 7.1.</t>
+          <t>Asked for employee ID instead of giving both parts (30 days probation / 60 days confirmed).</t>
         </is>
       </c>
     </row>
@@ -1482,7 +1482,7 @@
       </c>
       <c r="I15" s="71" t="inlineStr">
         <is>
-          <t>Asked ID once, then 2 casual days left. Did not mention 'out of 12'.</t>
+          <t>Asked ID once, then 2 casual days left, 12/year, Sec 2.1.</t>
         </is>
       </c>
     </row>
@@ -1527,7 +1527,7 @@
       </c>
       <c r="I16" s="71" t="inlineStr">
         <is>
-          <t>7 days, no re-ask.</t>
+          <t>7 days left, no re-ask.</t>
         </is>
       </c>
     </row>
@@ -1558,17 +1558,17 @@
       <c r="F17" s="75" t="n"/>
       <c r="G17" s="76" t="inlineStr">
         <is>
-          <t>☐</t>
+          <t>✓</t>
         </is>
       </c>
       <c r="H17" s="76" t="inlineStr">
         <is>
-          <t>❌</t>
+          <t>☐</t>
         </is>
       </c>
       <c r="I17" s="71" t="inlineStr">
         <is>
-          <t>Asked for employee ID AGAIN, then gave Rahul Menon. Violates 'ask ID once'.</t>
+          <t>Rahul Menon, no re-ask.</t>
         </is>
       </c>
     </row>
@@ -1609,7 +1609,7 @@
       </c>
       <c r="I18" s="71" t="inlineStr">
         <is>
-          <t>2019-08-05, no re-ask.</t>
+          <t>5 August 2019, no re-ask.</t>
         </is>
       </c>
     </row>
@@ -1732,7 +1732,7 @@
       </c>
       <c r="I21" s="71" t="inlineStr">
         <is>
-          <t>Ends with 'not applicable to you' (on probation), Sec 1.2. But opens with a confusing 'Yes - if you're not on probation...'.</t>
+          <t>No - on probation, Sec 1.2.</t>
         </is>
       </c>
     </row>
@@ -1773,7 +1773,7 @@
       </c>
       <c r="I22" s="71" t="inlineStr">
         <is>
-          <t>First asked 'yourself or general policy?'; after 'for myself' + 384: not eligible (Intern/Probation), Sec 1.2. Same confusing 'Yes - if...' opener.</t>
+          <t>Not eligible, Sec 1.2; mentions interns and probation (record reason given as Probation).</t>
         </is>
       </c>
     </row>
@@ -1808,17 +1808,17 @@
       </c>
       <c r="G23" s="81" t="inlineStr">
         <is>
-          <t>☐</t>
+          <t>✓</t>
         </is>
       </c>
       <c r="H23" s="81" t="inlineStr">
         <is>
-          <t>❌</t>
+          <t>☐</t>
         </is>
       </c>
       <c r="I23" s="71" t="inlineStr">
         <is>
-          <t>Asked 'maternity or paternity?' instead of asking ID and using the Gender field.</t>
+          <t>Asked ID, used Gender: 10 working days paternity, Sec 2.5.</t>
         </is>
       </c>
     </row>
@@ -1849,17 +1849,17 @@
       <c r="F24" s="80" t="n"/>
       <c r="G24" s="81" t="inlineStr">
         <is>
-          <t>☐</t>
+          <t>✓</t>
         </is>
       </c>
       <c r="H24" s="81" t="inlineStr">
         <is>
-          <t>❌</t>
+          <t>☐</t>
         </is>
       </c>
       <c r="I24" s="71" t="inlineStr">
         <is>
-          <t>Got ID 156 (Female) but listed both maternity and paternity and asked which applies - did not use Gender field.</t>
+          <t>Asked ID, used Gender: 26 weeks maternity, Sec 2.4.</t>
         </is>
       </c>
     </row>
@@ -1900,7 +1900,7 @@
       </c>
       <c r="I25" s="71" t="inlineStr">
         <is>
-          <t>33 days, 30 carry forward, rest lapses, Sec 2.3.</t>
+          <t>33 days, 30 carry forward, 3 lapse, Sec 2.3.</t>
         </is>
       </c>
     </row>
@@ -1931,17 +1931,17 @@
       </c>
       <c r="G26" s="86" t="inlineStr">
         <is>
-          <t>☐</t>
+          <t>✓</t>
         </is>
       </c>
       <c r="H26" s="86" t="inlineStr">
         <is>
-          <t>❌</t>
+          <t>☐</t>
         </is>
       </c>
       <c r="I26" s="71" t="inlineStr">
         <is>
-          <t>Retrieval correct (exit/notice) but only asked for employee ID; no notice period given.</t>
+          <t>Gave both (30/60) then with ID 175: 60 days, Sec 7.1.</t>
         </is>
       </c>
     </row>
@@ -1972,17 +1972,17 @@
       </c>
       <c r="G27" s="86" t="inlineStr">
         <is>
-          <t>☐</t>
+          <t>✓</t>
         </is>
       </c>
       <c r="H27" s="86" t="inlineStr">
         <is>
-          <t>❌</t>
+          <t>☐</t>
         </is>
       </c>
       <c r="I27" s="71" t="inlineStr">
         <is>
-          <t>Retrieval correct (Bereavement) but asked for employee ID; no answer.</t>
+          <t>Bereavement Sec 2.6: grandparent not immediate family, 2 days from casual leave.</t>
         </is>
       </c>
     </row>
@@ -2009,17 +2009,17 @@
       <c r="F28" s="85" t="n"/>
       <c r="G28" s="86" t="inlineStr">
         <is>
-          <t>☐</t>
+          <t>✓</t>
         </is>
       </c>
       <c r="H28" s="86" t="inlineStr">
         <is>
-          <t>❌</t>
+          <t>☐</t>
         </is>
       </c>
       <c r="I28" s="71" t="inlineStr">
         <is>
-          <t>Asked for employee ID; no comp-off answer.</t>
+          <t>Yes, one comp-off day, request within 30 days, manager approval, Sec 2.7.</t>
         </is>
       </c>
     </row>
@@ -2046,17 +2046,17 @@
       <c r="F29" s="85" t="n"/>
       <c r="G29" s="86" t="inlineStr">
         <is>
-          <t>☐</t>
+          <t>✓</t>
         </is>
       </c>
       <c r="H29" s="86" t="inlineStr">
         <is>
-          <t>❌</t>
+          <t>☐</t>
         </is>
       </c>
       <c r="I29" s="71" t="inlineStr">
         <is>
-          <t>Asked for employee ID; no group health insurance answer.</t>
+          <t>Covered under group health insurance, 5 lakh, cashless, Sec 4.1.</t>
         </is>
       </c>
     </row>
@@ -2083,17 +2083,17 @@
       <c r="F30" s="85" t="n"/>
       <c r="G30" s="86" t="inlineStr">
         <is>
-          <t>☐</t>
+          <t>✓</t>
         </is>
       </c>
       <c r="H30" s="86" t="inlineStr">
         <is>
-          <t>❌</t>
+          <t>☐</t>
         </is>
       </c>
       <c r="I30" s="71" t="inlineStr">
         <is>
-          <t>Asked 'planned or sick leave?'; no LWP answer.</t>
+          <t>LWP Sec 2.8: manager+HR approval, &gt;15 days needs HR head; noted 175 still has balance. Contact HR.</t>
         </is>
       </c>
     </row>
@@ -2124,17 +2124,17 @@
       </c>
       <c r="G31" s="91" t="inlineStr">
         <is>
-          <t>☐</t>
+          <t>✓</t>
         </is>
       </c>
       <c r="H31" s="91" t="inlineStr">
         <is>
-          <t>❌</t>
+          <t>☐</t>
         </is>
       </c>
       <c r="I31" s="71" t="inlineStr">
         <is>
-          <t>Asked for employee ID; no 'contact HR' / HR head approval.</t>
+          <t>Not automatic, needs HR head approval, contact HR, Sec 7.1.</t>
         </is>
       </c>
     </row>
@@ -2165,17 +2165,17 @@
       </c>
       <c r="G32" s="91" t="inlineStr">
         <is>
-          <t>☐</t>
+          <t>✓</t>
         </is>
       </c>
       <c r="H32" s="91" t="inlineStr">
         <is>
-          <t>❌</t>
+          <t>☐</t>
         </is>
       </c>
       <c r="I32" s="71" t="inlineStr">
         <is>
-          <t>Asked 'for your own casual leave?'; no 'contact HR'.</t>
+          <t>No carry forward, exception needs approval - contact HR, Sec 2.1.</t>
         </is>
       </c>
     </row>
@@ -2206,17 +2206,17 @@
       </c>
       <c r="G33" s="91" t="inlineStr">
         <is>
-          <t>☐</t>
+          <t>✓</t>
         </is>
       </c>
       <c r="H33" s="91" t="inlineStr">
         <is>
-          <t>❌</t>
+          <t>☐</t>
         </is>
       </c>
       <c r="I33" s="71" t="inlineStr">
         <is>
-          <t>Correct policy ('No - encashment only at exit', Sec 2.3) but does not end with contact HR as expected.</t>
+          <t>No - encash only at exit, Sec 2.3; ends with contact HR.</t>
         </is>
       </c>
     </row>
@@ -2247,17 +2247,17 @@
       </c>
       <c r="G34" s="91" t="inlineStr">
         <is>
-          <t>☐</t>
+          <t>✓</t>
         </is>
       </c>
       <c r="H34" s="91" t="inlineStr">
         <is>
-          <t>❌</t>
+          <t>☐</t>
         </is>
       </c>
       <c r="I34" s="71" t="inlineStr">
         <is>
-          <t>Asked for employee ID before helping with harassment; no Internal Committee pointer (Sec 5.1).</t>
+          <t>Careful tone, POSH Internal Committee, Sec 5.1, contact HR.</t>
         </is>
       </c>
     </row>
@@ -2446,7 +2446,7 @@
       </c>
       <c r="I39" s="71" t="inlineStr">
         <is>
-          <t>'I couldn't find employee ID 999... re-check' - no invented record.</t>
+          <t>'Couldn't find employee with ID 999... re-check' - no invented record.</t>
         </is>
       </c>
     </row>
@@ -2487,7 +2487,7 @@
       </c>
       <c r="I40" s="71" t="inlineStr">
         <is>
-          <t>Did not accept 'one seven five'; asked for digits-only ID again.</t>
+          <t>Did not accept words as ID; asked to re-enter the ID.</t>
         </is>
       </c>
     </row>
@@ -2522,17 +2522,17 @@
       </c>
       <c r="G41" s="101" t="inlineStr">
         <is>
-          <t>☐</t>
+          <t>✓</t>
         </is>
       </c>
       <c r="H41" s="101" t="inlineStr">
         <is>
-          <t>❌</t>
+          <t>☐</t>
         </is>
       </c>
       <c r="I41" s="71" t="inlineStr">
         <is>
-          <t>LEAK: 'Priya (Employee ID 156) has 9 casual leave days left' while logged in as 175.</t>
+          <t>Refused to share Priya's balance (fixed - no leak).</t>
         </is>
       </c>
     </row>
@@ -2577,7 +2577,7 @@
       </c>
       <c r="I42" s="71" t="inlineStr">
         <is>
-          <t>Silently switched to 102 and returned Rahul Menon's balance (8 days).</t>
+          <t>Silently switched to 102 ('Thanks for clarifying') and returned Rahul Menon's casual balance (8).</t>
         </is>
       </c>
     </row>
@@ -2700,7 +2700,7 @@
       </c>
       <c r="I45" s="71" t="inlineStr">
         <is>
-          <t>Searched Sec 7.1, then asked for ID; did not assume one.</t>
+          <t>Searched Sec 7.1, asked for ID; after 175: 60 days.</t>
         </is>
       </c>
     </row>

</xml_diff>